<commit_message>
Deployed 0cda087 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/data/indicator_data_export.xlsx
+++ b/data/indicator_data_export.xlsx
@@ -11,9 +11,9 @@
     <sheet name="Indicators" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="IndicatorCategories" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="IndicatorDataCollectionDetails" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Databases" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="IndicatorCriteria" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="IndicatorCriteriaScores" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="IndicatorCriteria" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="IndicatorCriteriaScores" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="ReferencesTab" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="IndicatorMeasurementUnit" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="SustainabilityDimension" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="FoodSystemActivityType" sheetId="10" state="visible" r:id="rId10"/>
@@ -26,6 +26,7 @@
     <sheet name="ScoreCategory" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="SustainabilityImpactType" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Eu2025SdgIndicator" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="ReferenceType" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,7 +465,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>The category the indicator belongs to.</t>
+          <t>Group of indicators that share common characteristics, functions, or measurement purposes within a monitoring or  evaluation framework.</t>
         </is>
       </c>
     </row>
@@ -481,7 +482,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A quantitative measure used to assess the state, performance, or progress of a specific aspect of the food system in relation to sustainability objectives.</t>
+          <t>A quantitative measure used to assess the state, performance, or progress of a specific aspect of the food system  in relation to sustainability objectives.</t>
         </is>
       </c>
     </row>
@@ -505,289 +506,323 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Database</t>
+          <t>IndicatorDatapoint</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>database</t>
+          <t>indicator datapoint</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Database containing data corresponding to an indicator.</t>
+          <t>A food system indicator datapoint is a measured value or statistic that provides quantitative information for a specific sustainability indicator at a given time and place, used to track the performance or state of the food system.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>IndicatorDatapoint</t>
+          <t>QuantityValue</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>indicator datapoint</t>
+          <t>quantity value</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>A food system indicator datapoint is a measured value or statistic that provides quantitative information for a specific sustainability indicator at a given time and place, used to track the performance or state of the food system.</t>
+          <t>A value of an attribute that is quantitative and measurable, expressed as a combination of a unit and a numeric value.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>QuantityValue</t>
+          <t>IndicatorCriterion</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>quantity value</t>
+          <t>indicator criterion</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A value of an attribute that is quantitative and measurable, expressed as a combination of a unit and a numeric value</t>
+          <t>Criterion used for indicator selection.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IndicatorCriterion</t>
+          <t>IndicatorcriteriaScore</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>indicator criterion</t>
+          <t>indicator criterion score</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Criterion used for indicator selection.</t>
+          <t>A score assigned to an indicator based on a specific selection criterion.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IndicatorcriteriaScore</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>indicator criterion score</t>
+          <t>reference</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Score for an indicator for an indicator selection criterion.</t>
+          <t>A reference to a publication, database or dataset.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>IndicatorMeasurementUnit</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Eurostat unit of measurement</t>
+          <t>database</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Food system indicator units of measurement imported from the Eurostat unit of measure dictionary/vocabulary.</t>
+          <t>A reference to a database.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SustainabilityDimension</t>
+          <t>IndicatorMeasurementUnit</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>sustainability dimension</t>
+          <t>Eurostat unit of measurement</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TODO</t>
+          <t>Food system indicator units of measurement imported from the Eurostat unit of measure dictionary/vocabulary.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FoodSystemActivityType</t>
+          <t>SustainabilityDimension</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>food system activity</t>
+          <t>sustainability dimension</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Food systems encompass  activities related to the food supply chains,  food environments, and food demand, as well as the use of natural resource, consumption and diets, and waste, by-products and recycling. These ultimately have an effect on  food system outcomes.</t>
+          <t>A dimension of sustainability to which the indicator relates.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>FoodSystemOutcomeType</t>
+          <t>FoodSystemActivityType</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>food system outcome</t>
+          <t>food system activity</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Food system outcomes, being impact related to environment, economic, social and health,  are a result of food systems. This framework distinguishes five different type of food system impacts: environmental, economic, social, health, and the overarching food security and resilience.</t>
+          <t>Food systems encompass  activities related to the food supply chains,  food environments, and food demand, as well as the use of natural resource, consumption and diets, and waste, by-products and recycling. These ultimately have an effect on  food system outcomes.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SpatialScopeType</t>
+          <t>FoodSystemOutcomeType</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>spatial scope type</t>
+          <t>food system outcome</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>The spatial scope for which the indicator is defined.</t>
+          <t>Food system outcomes, being impact related to environment, economic, social and health,  are a result of food systems. This framework distinguishes five different type of food system impacts: environmental, economic, social, health, and the overarching food security and resilience.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SupplyChainComponentType</t>
+          <t>SpatialScopeType</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>supply chain component type</t>
+          <t>spatial scope type</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>The supply chain component for which the indicator is relevant.</t>
+          <t>The spatial scope for which the indicator is defined.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TimeGranularity</t>
+          <t>SupplyChainComponentType</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>time granularity</t>
+          <t>supply chain component type</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Time granularity for measuring and updating data.</t>
+          <t>The supply chain component for which the indicator is relevant.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SpatialGranularity</t>
+          <t>TimeGranularity</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>spatial granularity</t>
+          <t>time granularity</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>The granularity for which the indicator is measured.</t>
+          <t>Time granularity for measuring and updating data.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CriterionCategory</t>
+          <t>SpatialGranularity</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>criterion category</t>
+          <t>spatial granularity</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Category of an indicator selection criterion.</t>
+          <t>The granularity for which the indicator is measured.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ScoreCategory</t>
+          <t>CriterionCategory</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>score category</t>
+          <t>criterion category</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Score category</t>
+          <t>Category of an indicator selection criterion.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SustainabilityImpactType</t>
+          <t>ScoreCategory</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>sustainability impact type</t>
+          <t>score category</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>The type of sustainability impact the indicator measures.</t>
+          <t>Score category.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>SustainabilityImpactType</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>sustainability impact type</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>The type of sustainability impact the indicator measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Eu2025SdgIndicator</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>EU SDG indicators</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Indicators of the 2025 edition of the EU sustainable development goals (SDG) monitoring report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ReferenceType</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Reference types</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>The type of source that a reference refers to.</t>
         </is>
       </c>
     </row>
@@ -7069,7 +7104,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -7124,7 +7159,7 @@
       </c>
       <c r="J106" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K106" t="inlineStr">
@@ -7175,7 +7210,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -7226,7 +7261,7 @@
       </c>
       <c r="J108" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K108" t="inlineStr">
@@ -7277,7 +7312,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -7328,7 +7363,7 @@
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K110" t="inlineStr">
@@ -7379,7 +7414,7 @@
       </c>
       <c r="J111" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K111" t="inlineStr">
@@ -7430,7 +7465,7 @@
       </c>
       <c r="J112" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K112" t="inlineStr">
@@ -7481,7 +7516,7 @@
       </c>
       <c r="J113" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K113" t="inlineStr">
@@ -7532,7 +7567,7 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
@@ -7583,7 +7618,7 @@
       </c>
       <c r="J115" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K115" t="inlineStr">
@@ -7634,7 +7669,7 @@
       </c>
       <c r="J116" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K116" t="inlineStr">
@@ -7685,7 +7720,7 @@
       </c>
       <c r="J117" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K117" t="inlineStr">
@@ -7736,7 +7771,7 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K118" t="inlineStr">
@@ -7787,7 +7822,7 @@
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -7838,7 +7873,7 @@
       </c>
       <c r="J120" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K120" t="inlineStr">
@@ -7889,7 +7924,7 @@
       </c>
       <c r="J121" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K121" t="inlineStr">
@@ -7940,7 +7975,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K122" t="inlineStr">
@@ -7991,7 +8026,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K123" t="inlineStr">
@@ -8042,7 +8077,7 @@
       </c>
       <c r="J124" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K124" t="inlineStr">
@@ -8093,7 +8128,7 @@
       </c>
       <c r="J125" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K125" t="inlineStr">
@@ -8144,7 +8179,7 @@
       </c>
       <c r="J126" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K126" t="inlineStr">
@@ -8195,7 +8230,7 @@
       </c>
       <c r="J127" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K127" t="inlineStr">
@@ -8246,7 +8281,7 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
@@ -8297,7 +8332,7 @@
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
@@ -8348,7 +8383,7 @@
       </c>
       <c r="J130" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K130" t="inlineStr">
@@ -8399,7 +8434,7 @@
       </c>
       <c r="J131" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K131" t="inlineStr">
@@ -8450,7 +8485,7 @@
       </c>
       <c r="J132" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K132" t="inlineStr">
@@ -8501,7 +8536,7 @@
       </c>
       <c r="J133" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K133" t="inlineStr">
@@ -8552,7 +8587,7 @@
       </c>
       <c r="J134" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K134" t="inlineStr">
@@ -8603,7 +8638,7 @@
       </c>
       <c r="J135" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K135" t="inlineStr">
@@ -8654,7 +8689,7 @@
       </c>
       <c r="J136" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K136" t="inlineStr">
@@ -8705,7 +8740,7 @@
       </c>
       <c r="J137" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K137" t="inlineStr">
@@ -8756,7 +8791,7 @@
       </c>
       <c r="J138" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="K138" t="inlineStr">
@@ -8807,7 +8842,7 @@
       </c>
       <c r="J139" t="inlineStr">
         <is>
-          <t>FoodQualitySafety</t>
+          <t>FoodQualityAndSafety</t>
         </is>
       </c>
       <c r="K139" t="inlineStr">
@@ -8862,7 +8897,7 @@
       </c>
       <c r="J140" t="inlineStr">
         <is>
-          <t>FoodQualitySafety</t>
+          <t>FoodQualityAndSafety</t>
         </is>
       </c>
       <c r="K140" t="inlineStr">
@@ -8913,7 +8948,7 @@
       </c>
       <c r="J141" t="inlineStr">
         <is>
-          <t>FoodQualitySafety</t>
+          <t>FoodQualityAndSafety</t>
         </is>
       </c>
       <c r="K141" t="inlineStr">
@@ -8964,7 +8999,7 @@
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>FoodQualitySafety</t>
+          <t>FoodQualityAndSafety</t>
         </is>
       </c>
       <c r="K142" t="inlineStr">
@@ -9015,7 +9050,7 @@
       </c>
       <c r="J143" t="inlineStr">
         <is>
-          <t>FoodQualitySafety</t>
+          <t>FoodQualityAndSafety</t>
         </is>
       </c>
       <c r="K143" t="inlineStr">
@@ -9066,7 +9101,7 @@
       </c>
       <c r="J144" t="inlineStr">
         <is>
-          <t>Malnutrition</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K144" t="inlineStr">
@@ -9117,7 +9152,7 @@
       </c>
       <c r="J145" t="inlineStr">
         <is>
-          <t>Malnutrition</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="K145" t="inlineStr">
@@ -9168,7 +9203,7 @@
       </c>
       <c r="J146" t="inlineStr">
         <is>
-          <t>FoodAccess</t>
+          <t>FoodSecurityAccessAndEnablingFactors</t>
         </is>
       </c>
       <c r="K146" t="inlineStr">
@@ -9219,7 +9254,7 @@
       </c>
       <c r="J147" t="inlineStr">
         <is>
-          <t>FoodAccess</t>
+          <t>FoodSecurityAccessAndEnablingFactors</t>
         </is>
       </c>
       <c r="K147" t="inlineStr">
@@ -9270,7 +9305,7 @@
       </c>
       <c r="J148" t="inlineStr">
         <is>
-          <t>FoodAccess</t>
+          <t>FoodSecurityAccessAndEnablingFactors</t>
         </is>
       </c>
       <c r="K148" t="inlineStr">
@@ -9321,7 +9356,7 @@
       </c>
       <c r="J149" t="inlineStr">
         <is>
-          <t>FoodAccess</t>
+          <t>FoodSecurityAccessAndEnablingFactors</t>
         </is>
       </c>
       <c r="K149" t="inlineStr">
@@ -9372,7 +9407,7 @@
       </c>
       <c r="J150" t="inlineStr">
         <is>
-          <t>FoodAccess</t>
+          <t>FoodSecurityAccessAndEnablingFactors</t>
         </is>
       </c>
       <c r="K150" t="inlineStr">
@@ -11591,6 +11626,68 @@
       </c>
       <c r="L193" t="inlineStr"/>
       <c r="M193" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Dataset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Publication.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -11603,7 +11700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11629,6 +11726,21 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>outcome_type</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>activity_type</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>referenced_in</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>iri</t>
         </is>
       </c>
@@ -11651,6 +11763,9 @@
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -11670,6 +11785,9 @@
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -11689,6 +11807,9 @@
         </is>
       </c>
       <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -11708,6 +11829,9 @@
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -11727,6 +11851,9 @@
         </is>
       </c>
       <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -11746,6 +11873,9 @@
         </is>
       </c>
       <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -11765,6 +11895,9 @@
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11784,6 +11917,9 @@
         </is>
       </c>
       <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11803,6 +11939,9 @@
         </is>
       </c>
       <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -11822,6 +11961,9 @@
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -11841,6 +11983,9 @@
         </is>
       </c>
       <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11860,6 +12005,9 @@
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11879,6 +12027,9 @@
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -11898,6 +12049,9 @@
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11917,6 +12071,9 @@
         </is>
       </c>
       <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11936,6 +12093,9 @@
         </is>
       </c>
       <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -11955,6 +12115,9 @@
         </is>
       </c>
       <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -11974,149 +12137,245 @@
         </is>
       </c>
       <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NutritionalHealthOutcomes</t>
+          <t>NutritionAndHealth</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nutritional health outcomes</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>Nutrition and Health</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Indicators capturing the final health outcomes of food systems, encompassing nutritional status and malnutrition in all its forms,  including undernutrition, micronutrient deficiencies, overweight, obesity, and diet-related non-communicable diseases.</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>['HLPE2017']</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NutritionalBehaviour</t>
+          <t>DietaryConsumptionPatternsFoodIntake</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nutritional behaviour</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr"/>
+          <t>Dietary consumption patterns/Food Intake</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Indicators describing the dietary consumption patterns refer to the quantities, proportions, and habitual combinations of foods and  drinks that individuals or populations.</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
       <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>ConsumptionAndDiets</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>['USDHHS2020']</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FoodQualitySafety</t>
+          <t>FoodQualityAndSafety</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Food quality &amp; safety</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr"/>
+          <t>Food quality and safety</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Indicators describing the extent to which foods meet established standards of safety and quality, including the absence of  biological, chemical, and physical hazards, as well as compliance with nutritional, compositional, and hygienic requirements  along the food chain.</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>['FAO2003']</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Malnutrition</t>
+          <t>FoodSecurityAccessAndEnablingFactors</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Malnutrition</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr"/>
+          <t>Food security: access and enabling factors</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Indicators capturing both people's ability to obtain adequate food (economic and physical access) and the broader economic,  infrastructural, and systemic conditions that enable or constrain such access.</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>FoodSecurity</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>['FAO2008']</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FoodAccess</t>
+          <t>FoodAvailability</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Food access</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr"/>
+          <t>Food availability</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Indicators describing the quantity, composition, and stability of food supplied by the food system through domestic production,  imports, and stocks, including the supply of energy and nutrients and the productive capacity of agriculture.</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
       <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>FoodEnvironment</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>['FAO2008']</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FoodAvailability</t>
+          <t>FoodStability</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Food availability</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr"/>
+          <t>Food stability</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Indicators describing the extent to which the availability of and access to food are maintained over time, including the  resilience of food supply systems to economic, climatic, and market-related shocks and variability.</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
           <t>Health</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Resilience</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>['FAO2008']</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FoodStability</t>
+          <t>EmploymInAgricFoodSector</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Food stability</t>
+          <t>Employm. in agric._food sector</t>
         </is>
       </c>
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Health</t>
+          <t>Society</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>EmploymInAgricFoodSector</t>
+          <t>WorkingCondAgricFoodSect</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Employm. in agric._food sector</t>
+          <t>Working cond._agric. food sect.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -12126,16 +12385,19 @@
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>WorkingCondAgricFoodSect</t>
+          <t>GeneralUnEmployment</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Working cond._agric. food sect.</t>
+          <t>General (un)employment</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -12145,16 +12407,19 @@
         </is>
       </c>
       <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>GeneralUnEmployment</t>
+          <t>IncomeDistributPovertyRisk</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>General (un)employment</t>
+          <t>Income distribut._Poverty risk</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -12164,16 +12429,19 @@
         </is>
       </c>
       <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IncomeDistributPovertyRisk</t>
+          <t>FoodEquity</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Income distribut._Poverty risk</t>
+          <t>Food Equity</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -12183,16 +12451,19 @@
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FoodEquity</t>
+          <t>GenderEquity</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Food Equity</t>
+          <t>Gender Equity</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -12202,16 +12473,19 @@
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GenderEquity</t>
+          <t>Demography</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Gender Equity</t>
+          <t>Demography</t>
         </is>
       </c>
       <c r="C32" t="inlineStr"/>
@@ -12221,16 +12495,19 @@
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Demography</t>
+          <t>SocialResilience</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Demography</t>
+          <t>Social resilience</t>
         </is>
       </c>
       <c r="C33" t="inlineStr"/>
@@ -12240,16 +12517,19 @@
         </is>
       </c>
       <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SocialResilience</t>
+          <t>RuralDevelopment</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Social resilience</t>
+          <t>Rural development</t>
         </is>
       </c>
       <c r="C34" t="inlineStr"/>
@@ -12259,25 +12539,9 @@
         </is>
       </c>
       <c r="E34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>RuralDevelopment</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Rural development</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr"/>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Society</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12624,7 +12888,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>AgriFoodDataPortalDirectorateGeneralForAgriculture</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -12974,7 +13238,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DataModellingPlatformOfResourceEconomicsJrcLasarte</t>
+          <t>DataModellingPlatformOfResourceEconomics</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -13024,7 +13288,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EuFoodSystemMonitoringDashboardJrc</t>
+          <t>DataModellingPlatformOfResourceEconomics</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -13074,7 +13338,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>AgriFoodDataPortalDirectorateGeneralForAgriculture</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -14424,7 +14688,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -16524,7 +16788,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F85" t="inlineStr"/>
@@ -16574,7 +16838,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F86" t="inlineStr"/>
@@ -16624,7 +16888,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F87" t="inlineStr"/>
@@ -16674,7 +16938,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F88" t="inlineStr"/>
@@ -16724,7 +16988,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F89" t="inlineStr"/>
@@ -16774,7 +17038,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F90" t="inlineStr"/>
@@ -16824,7 +17088,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F91" t="inlineStr"/>
@@ -16874,7 +17138,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F92" t="inlineStr"/>
@@ -16924,7 +17188,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F93" t="inlineStr"/>
@@ -16974,7 +17238,7 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F94" t="inlineStr"/>
@@ -17024,7 +17288,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F95" t="inlineStr"/>
@@ -17074,7 +17338,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F96" t="inlineStr"/>
@@ -17124,7 +17388,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F97" t="inlineStr"/>
@@ -17174,7 +17438,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F98" t="inlineStr"/>
@@ -17224,7 +17488,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F99" t="inlineStr"/>
@@ -17274,7 +17538,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
+          <t>AgriFoodDataPortal</t>
         </is>
       </c>
       <c r="F100" t="inlineStr"/>
@@ -17874,7 +18138,7 @@
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Who2024</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="F112" t="inlineStr"/>
@@ -18874,7 +19138,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Who2022</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="F132" t="inlineStr"/>
@@ -18924,7 +19188,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Who2022</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="F133" t="inlineStr"/>
@@ -18974,7 +19238,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Who2022</t>
+          <t>Who</t>
         </is>
       </c>
       <c r="F134" t="inlineStr"/>
@@ -20374,7 +20638,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>DataModellingPlatformOfResourceEconomicsJrcLasarte</t>
+          <t>DataModellingPlatformOfResourceEconomics</t>
         </is>
       </c>
       <c r="F162" t="inlineStr"/>
@@ -21566,36 +21830,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>database_link</t>
+          <t>category</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>update_frequency</t>
+          <t>rationale_strong</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>rationale_adequate</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rationale_weak</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>iri</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -21604,410 +21878,416 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://ec.europa.eu/eurostat/databrowser/view/sdg_01_10a/default/table?lang=en</t>
+          <t>CoherenceOnFramework</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Mapped once or multiple times; no redundancy.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Eurostat</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
+          <t>Mapped once or multiple times; partially redundancy.</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Mapped once or multiple times; redundancy.</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Eurostat</t>
+          <t>IntegrationFoodSystemFramework</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>integration on food system framework</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Integration on food system framework Indicators should be mapped within a food system framework and assessed as part of an integrated set, ensuring each provides a unique, non-redundant contribution. Collectively, they must offer a balanced and comprehensive representation of the food system. The operative allocation involves mapping indicators within the framework and maintaining system-level coherence to guarantee their relevance and effectiveness.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.fao.org/faostat/en/#data/OA</t>
+          <t>GoalOrientedAndPolicyRelevant</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>SDGs, Farm to Fork,.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Faostat</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
+          <t>Partially linked to sustainable objectives.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Not linked.</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>FAOSTAT</t>
+          <t>GoalAlignment</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>goal alignment</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Indicators should align with key sustainability frameworks (SDGs, Green Deal, Farm to Fork, national food policies) and should be clearly linked to relevant SRIA objectives providing a measurable signal of progress on the associated objective. Procedures should be in place to update the prioritization of indicators as SRIA priorities evolve, assessing whether any existing indicator can be adapted for the new purpose without altering what it measures. Any methodological changes should be documented, and if an indicator no longer fits, a new one should be created.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://agridata.ec.europa.eu/extensions/DashboardIndicators/AddingValue.html</t>
+          <t>GoalOrientedAndPolicyRelevant</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Behavioral indicators (e.g., frequency/consumption, interpretable direction).</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>AgriFoodDataPortalDirectorateGeneralForAgriculture</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>Outcome indicators (e.g., prevalences) that require complementary indicators to capture the mechanisms of transition.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No clear indication or outcome of the indicator.</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Agri-food data portal (Directorate-General for Agriculture and Rural Development)</t>
+          <t>TransitionMonitoring</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>transition monitoring</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Interpretability and evidence of transition. Indicators interoperability (OR INTERDEPENDENCY?? synergies) (need of definition) to identify the progress of transition. Clearly interpretable direction of food system transition with evidence of the outcomes (Fanzo 2023; EUROSTAT 2017</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://data.worldbank.org/indicator/PV.EST?view=chart</t>
+          <t>GoalOrientedAndPolicyRelevant</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Official datasets/statistics (interpretable and communicable to non-technical audiences.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>WorldBankGroup</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
+          <t>Individual studies when applicability for policy is more limited.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>No applicable for policy decision and no clear.</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>World Bank Group</t>
+          <t>DecisionUsefulness</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>decision-usefulness</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Indicators have to inform concrete policies and strategies for decision-makers (public authorities, policymakers, farmers, industry, and consumers) and have to be interpretable, Unambiguous  and communicable to a broad audience also for non-technical stakeholders.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://datam.jrc.ec.europa.eu/datam/mashup/BIOECONOMICS/</t>
+          <t>SoundMethodologies</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Databases/reports from international organizations.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DataModellingPlatformOfResourceEconomicsJrcLasarte</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
+          <t>Documentation is limited.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>No Documentation.</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Data-Modelling platform of resource economics (JRC) / Lasarte-López et al. (2023)</t>
+          <t>StandardizationComparabilityComplementarity</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>standardization, comparability, and complementarity</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Indicators should be based on international standards, harmonized definitions, and statistical methodologies to ensure comparability among countries. Adhering to such standards enhances the credibility of the data, facilitates integration into global monitoring frameworks, and allows meaningful cross-national benchmarking. This alignment also ensures that methodologies are transparent, replicable, and coherent with global best practices, strengthening the overall validity and utility of the indicators. Indicators should be assessed for interdependencies and complementarity, for example through interdependency mapping or interoperability analysis</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://datam.jrc.ec.europa.eu/datam/mashup/EU_FOOD_SYSTEM_MONITORING/index.html</t>
+          <t>SoundMethodologies</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Official datasets and for indicators supported by peer-reviewed literature.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>EuFoodSystemMonitoringDashboardJrc</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
+          <t>Documentation is limited.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>No Documentation.</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>EU Food System Monitoring Dashboard (JRC)</t>
+          <t>ScientificRigorAndValidation</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>scientific rigor and validation</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Indicators should be grounded in scientifically validated evidence and supported by peer-reviewed research to ensure methodological rigor and credibility. Reliance on peer-reviewed sources guarantees that data collection methods, analytical approaches, and interpretations have undergone critical evaluation by experts, enhancing transparency, reliability, and alignment with established scientific standards.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://datam.jrc.ec.europa.eu/datam/mashup/EU_ESTIMATED_AGRICULTURAL_BALANCE_SHEETS/</t>
+          <t>SoundMethodologies</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Recent data are available.</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DataModellingPlatformOfResourceEconomics</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
+          <t>Records indicate data gaps or the most recent year is old.</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>No recent or past data available.</t>
+        </is>
+      </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Data-Modelling platform of resource economics</t>
+          <t>DataAvailability</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>data availability</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Data availability, (existing of data (Findability), data availability refers to whether the required data exists and can be obtained for the indicator. It means the data has been collected, stored, and is present in some form (e.g., databases, reports, surveys)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://agridata.ec.europa.eu/extensions/DashboardCapPlan/result_indicators.html</t>
+          <t>SoundMethodologies</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>The link is public and direct.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cap202327ResultIndicatorsEuropeanCommissionDirecto</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>Partially accessible.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Not accessible.</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>CAP 2023 - 27: Result indicators (European Commission, Directorate-General for Agriculture and Rural Development)</t>
+          <t>DataAccessibility</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>data accessibility</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Data accessibility (Ease of obtaining data), data are accessible for different of aggregation level. Ensuring that data are publicly accessible aligns with the purpose of the indicator, which is to make data obtainable, usable, and understandable by all r stakeholders. If the data are available only internally or behind restricted access, they would not fully meet the criteria.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://esvacbi.ema.europa.eu/analytics/saw.dll?Dashboard</t>
+          <t>SoundMethodologies</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>Large integrable databases.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>EuropeanDatabaseOfSalesOfVeterinaryAntmicrobialAge</t>
+          <t>Partial interoperability or heterogeneous collections.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>European database of sales of veterinary antmicrobial agents (EMA)</t>
+          <t>DataInteroperability</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>data interoperability</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>The data should be easily integrated with other sources and information systems (Can the data work with other datasets?), and data could be used to develop to more than one indicator.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://agriculture.ec.europa.eu/farming/animal-products/eggs_en</t>
+          <t>GeographicalCoverageAndTimeliness</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Yearly</t>
+          <t>\&gt;=27.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DirectorateGeneralForAgricultureAndRuralDevelopmen</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>15-26.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>&lt;15.</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Directorate-General for Agriculture and Rural Development</t>
+          <t>BroadGeographicalCoverage</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>broad geographical coverage</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Indicators have to be based on data with broad geographical coverage (i.e., an indicator on agricultural GHG emissions should include data from both high-income and low-income countries). Data should be available at appropriate territorial scales (local, regional, national, and global), depending on the monitoring objectives.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://agridata.ec.europa.eu/extensions/IndicatorsSectorial/AgriculturalTrainingOfFarmManagers.html</t>
+          <t>GeographicalCoverageAndTimeliness</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>&lt;=1 year.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>AgriFoodDataPortal</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>2-3 years.</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>\&gt;3 years.</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Agri-food data portal</t>
+          <t>Timeliness</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>https://eplca.jrc.ec.europa.eu/ConsumptionFootprintPlatform.html</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Yearly</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>EcEuropeanPlatformOnLifeCycleAssessmentEplca</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>EC / European Platform on life cycle assessment (EPLCA)</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>https://www.who.int/europe/publications/m/item/brief-review-of-results-from-round-6-of-cosi-2022-2024</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Who2024</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>WHO (2024)</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>https://www.efsa.europa.eu/en/microstrategy/foodex2-level-3</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>EfsaComprehensiveEuropeanFoodConsumptionDatabase</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>EFSA Comprehensive European Food Consumption Database</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>https://www.sciencedirect.com/science/article/pii/S0959652619326873</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>MertensEtAl2019</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Mertens et al. (2019)</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>https://www.who.int/europe/publications/i/item/WHO-EURO-2022-6594-46360-67071</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Who2022</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>WHO (2022)</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>https://digital-decade-desi.digital-strategy.ec.europa.eu/datasets/key-indicators/charts/analyse-one-indicator-and-compare-countries?indicator=bb_rngacov&amp;indicatorGroup=broadband&amp;breakdown=total_pophh&amp;period=2022&amp;unit=pc_hh_all&amp;country=AT,BE,BG,HR,CY,CZ,DK,EE,EU,FI,FR,DE,EL,HU,IS,IE,IT,LV,LT,LU,MT,NL,NO,PL,PT,RO,SK,SI,ES,SE,UK</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Yearly</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>DirectorateGeneralForCommunicationsNetworksContent</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Directorate-General for Communications Networks, Content and Technology</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>timeliness</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Indicators should provide up-to-date and regularly updated data that accurately reflect the current state and performance of the sustainable food system. Timely data support early detection of trends, emerging issues, or progress, enabling informed decision-making. Updates should be frequent enough to be useful while maintaining data quality and consistency with other indicators for integrated analysis.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22020,40 +22300,35 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>score_for_indicator</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>scores_criterion</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>iri</t>
+          <t>score</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>description</t>
+          <t>comment</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CoherenceOnFramework</t>
+          <t>FSI_0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -22062,246 +22337,7 @@
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>integration on food system framework</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Integration on food system framework Indicators should be mapped within a food system framework and assessed as part of an integrated set, ensuring each provides a unique, non-redundant contribution. Collectively, they must offer a balanced and comprehensive representation of the food system. The operative allocation involves mapping indicators within the framework and maintaining system-level coherence to guarantee their relevance and effectiveness.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>GoalOrientedAndPolicyRelevant</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>GoalAlignment</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>goal alignment</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Indicators should align with key sustainability frameworks (SDGs, Green Deal, Farm to Fork, national food policies) and should be clearly linked to relevant SRIA objectives providing a measurable signal of progress on the associated objective. Procedures should be in place to update the prioritization of indicators as SRIA priorities evolve, assessing whether any existing indicator can be adapted for the new purpose without altering what it measures. Any methodological changes should be documented, and if an indicator no longer fits, a new one should be created.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>GoalOrientedAndPolicyRelevant</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>TransitionMonitoring</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>transition monitoring</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Interpretability and evidence of transition. Indicators interoperability (OR INTERDEPENDENCY?? synergies) (need of definition) to identify the progress of transition. Clearly interpretable direction of food system transition with evidence of the outcomes (Fanzo 2023; EUROSTAT 2017</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>GoalOrientedAndPolicyRelevant</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>DecitionUsefulness</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>decision-usefulness</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Indicators have to inform concrete policies and strategies for decision-makers (public authorities, policymakers, farmers, industry, and consumers) and have to be interpretable, Unambiguous  and communicable to a broad audience also for non-technical stakeholders.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>SoundMethodologies</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>StandardizationComparabilityComplementarity</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>standardization, comparability, and complementarity</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Indicators should be based on international standards, harmonized definitions, and statistical methodologies to ensure comparability among countries. Adhering to such standards enhances the credibility of the data, facilitates integration into global monitoring frameworks, and allows meaningful cross-national benchmarking. This alignment also ensures that methodologies are transparent, replicable, and coherent with global best practices, strengthening the overall validity and utility of the indicators. Indicators should be assessed for interdependencies and complementarity, for example through interdependency mapping or interoperability analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>SoundMethodologies</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ScientificRigorAndValidation</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>scientific rigor and validation</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Indicators should be grounded in scientifically validated evidence and supported by peer-reviewed research to ensure methodological rigor and credibility. Reliance on peer-reviewed sources guarantees that data collection methods, analytical approaches, and interpretations have undergone critical evaluation by experts, enhancing transparency, reliability, and alignment with established scientific standards.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>SoundMethodologies</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>DataAvailability</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>data availability</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Data availability, (existing of data (Findability), data availability refers to whether the required data exists and can be obtained for the indicator. It means the data has been collected, stored, and is present in some form (e.g., databases, reports, surveys)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>SoundMethodologies</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DataAccessibility</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>data accessibility</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Data accessibility (Ease of obtaining data), data are accessible for different of aggregation level. Ensuring that data are publicly accessible aligns with the purpose of the indicator, which is to make data obtainable, usable, and understandable by all r stakeholders. If the data are available only internally or behind restricted access, they would not fully meet the criteria.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>SoundMethodologies</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>DataInteroperability</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>data interoperability</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>The data should be easily integrated with other sources and information systems (Can the data work with other datasets?), and data could be used to develop to more than one indicator.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>GeographicalCoverageAndTimeliness</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>BroadGeographicalCoverage</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>broad geographical coverage</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Indicators have to be based on data with broad geographical coverage (i.e., an indicator on agricultural GHG emissions should include data from both high-income and low-income countries). Data should be available at appropriate territorial scales (local, regional, national, and global), depending on the monitoring objectives.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>GeographicalCoverageAndTimeliness</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Timeliness</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>timeliness</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Indicators should provide up-to-date and regularly updated data that accurately reflect the current state and performance of the sustainable food system. Timely data support early detection of trends, emerging issues, or progress, enabling informed decision-making. Updates should be frequent enough to be useful while maintaining data quality and consistency with other indicators for integrated analysis.</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -22314,44 +22350,445 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>score_for_indicator</t>
+          <t>link</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>scores_criterion</t>
+          <t>reference_type</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>score</t>
+          <t>comment</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>comment</t>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>iri</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>FSI_0001</t>
+          <t>https://ec.europa.eu/eurostat/</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IntegrationFoodSystemFramework</t>
+          <t>Database</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Eurostat</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Eurostat</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>https://www.fao.org/faostat/</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Faostat</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>FAOSTAT</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>https://agridata.ec.europa.eu/</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>AgriFoodDataPortal</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Agri-food data portal</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>https://data.worldbank.org/</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>WorldBankGroup</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>World Bank Group</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>https://datam.jrc.ec.europa.eu/</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>DataModellingPlatformOfResourceEconomics</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Data-Modelling platform of resource economics (JRC)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>https://esvacbi.ema.europa.eu/analytics/saw.dll?Dashboard</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>EuropeanDatabaseOfSalesOfVeterinaryAntmicrobialAge</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>European database of sales of veterinary antmicrobial agents (EMA)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>https://agriculture.ec.europa.eu/</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>DirectorateGeneralForAgricultureAndRuralDevelopmen</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Directorate-General for Agriculture and Rural Development</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>https://eplca.jrc.ec.europa.eu/</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>EcEuropeanPlatformOnLifeCycleAssessmentEplca</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>EC / European Platform on life cycle assessment (EPLCA)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>https://www.who.int/</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>WHO</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>https://www.efsa.europa.eu/</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>EfsaComprehensiveEuropeanFoodConsumptionDatabase</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>EFSA Comprehensive European Food Consumption Database</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>https://www.sciencedirect.com/science/article/pii/S0959652619326873</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MertensEtAl2019</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Mertens et al. (2019)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>https://digital-decade-desi.digital-strategy.ec.europa.eu/</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>DirectorateGeneralForCommunicationsNetworksContent</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Directorate-General for Communications Networks, Content and Technology</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>HLPE2017</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>HLPE 2017</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Nutrition and food systems. A report by the High Level Panel of Experts on Food Security and Nutrition of the Committee on World Food Security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>USDHHS2020</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>USDHHS 2020</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>U.S. Department of Health and Human Services &amp; U.S. Department of Agriculture (2020). Scientific Report of the 2020 Dietary  Guidelines Advisory Committee. Washington, DC: U.S. Government Printing Office.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FAO2003</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>FAO 2003</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Assuring Food Safety and Quality: Guidelines for Strengthening National Food Control System.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Publication</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FAO2008</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>FAO 2008</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Food and Agriculture Organization of the United Nations. An introduction to the basic concepts of food security.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Deployed 529db3c with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/data/indicator_data_export.xlsx
+++ b/data/indicator_data_export.xlsx
@@ -1733,7 +1733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M193"/>
+  <dimension ref="A1:N193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1799,6 +1799,11 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>methodology_description</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>iri</t>
         </is>
       </c>
@@ -1857,6 +1862,7 @@
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1908,6 +1914,7 @@
       </c>
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1959,6 +1966,7 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2010,6 +2018,7 @@
       </c>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2061,6 +2070,7 @@
       </c>
       <c r="L6" t="inlineStr"/>
       <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2112,6 +2122,7 @@
       </c>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2167,6 +2178,7 @@
         </is>
       </c>
       <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2222,6 +2234,7 @@
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2273,6 +2286,7 @@
       </c>
       <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2324,6 +2338,7 @@
       </c>
       <c r="L11" t="inlineStr"/>
       <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2375,6 +2390,7 @@
       </c>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2426,6 +2442,7 @@
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2477,6 +2494,7 @@
       </c>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2528,6 +2546,7 @@
       </c>
       <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2579,6 +2598,7 @@
       </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2630,6 +2650,7 @@
       </c>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2681,6 +2702,7 @@
       </c>
       <c r="L18" t="inlineStr"/>
       <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2732,6 +2754,7 @@
       </c>
       <c r="L19" t="inlineStr"/>
       <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2783,6 +2806,7 @@
       </c>
       <c r="L20" t="inlineStr"/>
       <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2834,6 +2858,7 @@
       </c>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2885,6 +2910,7 @@
       </c>
       <c r="L22" t="inlineStr"/>
       <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2936,6 +2962,7 @@
       </c>
       <c r="L23" t="inlineStr"/>
       <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2987,6 +3014,7 @@
       </c>
       <c r="L24" t="inlineStr"/>
       <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3038,6 +3066,7 @@
       </c>
       <c r="L25" t="inlineStr"/>
       <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3089,6 +3118,7 @@
       </c>
       <c r="L26" t="inlineStr"/>
       <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3140,6 +3170,7 @@
       </c>
       <c r="L27" t="inlineStr"/>
       <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3191,6 +3222,7 @@
       </c>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3242,6 +3274,7 @@
       </c>
       <c r="L29" t="inlineStr"/>
       <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3293,6 +3326,7 @@
       </c>
       <c r="L30" t="inlineStr"/>
       <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3348,6 +3382,7 @@
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3403,6 +3438,7 @@
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3454,6 +3490,7 @@
       </c>
       <c r="L33" t="inlineStr"/>
       <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3505,6 +3542,7 @@
       </c>
       <c r="L34" t="inlineStr"/>
       <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3556,6 +3594,7 @@
       </c>
       <c r="L35" t="inlineStr"/>
       <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3607,6 +3646,7 @@
       </c>
       <c r="L36" t="inlineStr"/>
       <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3654,6 +3694,7 @@
       </c>
       <c r="L37" t="inlineStr"/>
       <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3705,6 +3746,7 @@
       </c>
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3756,6 +3798,7 @@
       </c>
       <c r="L39" t="inlineStr"/>
       <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3807,6 +3850,7 @@
       </c>
       <c r="L40" t="inlineStr"/>
       <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3858,6 +3902,7 @@
       </c>
       <c r="L41" t="inlineStr"/>
       <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3909,6 +3954,7 @@
       </c>
       <c r="L42" t="inlineStr"/>
       <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3960,6 +4006,7 @@
       </c>
       <c r="L43" t="inlineStr"/>
       <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4015,6 +4062,7 @@
         </is>
       </c>
       <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4062,6 +4110,7 @@
       </c>
       <c r="L45" t="inlineStr"/>
       <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4109,6 +4158,7 @@
       </c>
       <c r="L46" t="inlineStr"/>
       <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4160,6 +4210,7 @@
       </c>
       <c r="L47" t="inlineStr"/>
       <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4211,6 +4262,7 @@
       </c>
       <c r="L48" t="inlineStr"/>
       <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4262,6 +4314,7 @@
       </c>
       <c r="L49" t="inlineStr"/>
       <c r="M49" t="inlineStr"/>
+      <c r="N49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4313,6 +4366,7 @@
       </c>
       <c r="L50" t="inlineStr"/>
       <c r="M50" t="inlineStr"/>
+      <c r="N50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4364,6 +4418,7 @@
       </c>
       <c r="L51" t="inlineStr"/>
       <c r="M51" t="inlineStr"/>
+      <c r="N51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4415,6 +4470,7 @@
       </c>
       <c r="L52" t="inlineStr"/>
       <c r="M52" t="inlineStr"/>
+      <c r="N52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4466,6 +4522,7 @@
       </c>
       <c r="L53" t="inlineStr"/>
       <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4521,6 +4578,7 @@
         </is>
       </c>
       <c r="M54" t="inlineStr"/>
+      <c r="N54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4572,6 +4630,7 @@
       </c>
       <c r="L55" t="inlineStr"/>
       <c r="M55" t="inlineStr"/>
+      <c r="N55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4623,6 +4682,7 @@
       </c>
       <c r="L56" t="inlineStr"/>
       <c r="M56" t="inlineStr"/>
+      <c r="N56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4674,6 +4734,7 @@
       </c>
       <c r="L57" t="inlineStr"/>
       <c r="M57" t="inlineStr"/>
+      <c r="N57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4725,6 +4786,7 @@
       </c>
       <c r="L58" t="inlineStr"/>
       <c r="M58" t="inlineStr"/>
+      <c r="N58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4776,6 +4838,7 @@
       </c>
       <c r="L59" t="inlineStr"/>
       <c r="M59" t="inlineStr"/>
+      <c r="N59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -4827,6 +4890,7 @@
       </c>
       <c r="L60" t="inlineStr"/>
       <c r="M60" t="inlineStr"/>
+      <c r="N60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4878,6 +4942,7 @@
       </c>
       <c r="L61" t="inlineStr"/>
       <c r="M61" t="inlineStr"/>
+      <c r="N61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4929,6 +4994,7 @@
       </c>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
+      <c r="N62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4980,6 +5046,7 @@
       </c>
       <c r="L63" t="inlineStr"/>
       <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5031,6 +5098,7 @@
       </c>
       <c r="L64" t="inlineStr"/>
       <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5082,6 +5150,7 @@
       </c>
       <c r="L65" t="inlineStr"/>
       <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5137,6 +5206,7 @@
         </is>
       </c>
       <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5188,6 +5258,7 @@
       </c>
       <c r="L67" t="inlineStr"/>
       <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5239,6 +5310,7 @@
       </c>
       <c r="L68" t="inlineStr"/>
       <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5290,6 +5362,7 @@
       </c>
       <c r="L69" t="inlineStr"/>
       <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5341,6 +5414,7 @@
       </c>
       <c r="L70" t="inlineStr"/>
       <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5392,6 +5466,7 @@
       </c>
       <c r="L71" t="inlineStr"/>
       <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5443,6 +5518,7 @@
       </c>
       <c r="L72" t="inlineStr"/>
       <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5494,6 +5570,7 @@
       </c>
       <c r="L73" t="inlineStr"/>
       <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5545,6 +5622,7 @@
       </c>
       <c r="L74" t="inlineStr"/>
       <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5596,6 +5674,7 @@
       </c>
       <c r="L75" t="inlineStr"/>
       <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5647,6 +5726,7 @@
       </c>
       <c r="L76" t="inlineStr"/>
       <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5698,6 +5778,7 @@
       </c>
       <c r="L77" t="inlineStr"/>
       <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -5753,6 +5834,7 @@
         </is>
       </c>
       <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5800,6 +5882,7 @@
       </c>
       <c r="L79" t="inlineStr"/>
       <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5847,6 +5930,7 @@
       </c>
       <c r="L80" t="inlineStr"/>
       <c r="M80" t="inlineStr"/>
+      <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5894,6 +5978,7 @@
       </c>
       <c r="L81" t="inlineStr"/>
       <c r="M81" t="inlineStr"/>
+      <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5945,6 +6030,7 @@
       </c>
       <c r="L82" t="inlineStr"/>
       <c r="M82" t="inlineStr"/>
+      <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5992,6 +6078,7 @@
       </c>
       <c r="L83" t="inlineStr"/>
       <c r="M83" t="inlineStr"/>
+      <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6043,6 +6130,7 @@
       </c>
       <c r="L84" t="inlineStr"/>
       <c r="M84" t="inlineStr"/>
+      <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6094,6 +6182,7 @@
       </c>
       <c r="L85" t="inlineStr"/>
       <c r="M85" t="inlineStr"/>
+      <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6145,6 +6234,7 @@
       </c>
       <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr"/>
+      <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6196,6 +6286,7 @@
       </c>
       <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr"/>
+      <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6247,6 +6338,7 @@
       </c>
       <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr"/>
+      <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6298,6 +6390,7 @@
       </c>
       <c r="L89" t="inlineStr"/>
       <c r="M89" t="inlineStr"/>
+      <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6349,6 +6442,7 @@
       </c>
       <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr"/>
+      <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6400,6 +6494,7 @@
       </c>
       <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr"/>
+      <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6451,6 +6546,7 @@
       </c>
       <c r="L92" t="inlineStr"/>
       <c r="M92" t="inlineStr"/>
+      <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6502,6 +6598,7 @@
       </c>
       <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr"/>
+      <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6553,6 +6650,7 @@
       </c>
       <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr"/>
+      <c r="N94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6604,6 +6702,7 @@
       </c>
       <c r="L95" t="inlineStr"/>
       <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -6655,6 +6754,7 @@
       </c>
       <c r="L96" t="inlineStr"/>
       <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -6706,6 +6806,7 @@
       </c>
       <c r="L97" t="inlineStr"/>
       <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -6757,6 +6858,7 @@
       </c>
       <c r="L98" t="inlineStr"/>
       <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -6808,6 +6910,7 @@
       </c>
       <c r="L99" t="inlineStr"/>
       <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -6859,6 +6962,7 @@
       </c>
       <c r="L100" t="inlineStr"/>
       <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -6910,6 +7014,7 @@
       </c>
       <c r="L101" t="inlineStr"/>
       <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -6961,6 +7066,7 @@
       </c>
       <c r="L102" t="inlineStr"/>
       <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7012,6 +7118,7 @@
       </c>
       <c r="L103" t="inlineStr"/>
       <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7063,6 +7170,7 @@
       </c>
       <c r="L104" t="inlineStr"/>
       <c r="M104" t="inlineStr"/>
+      <c r="N104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7118,6 +7226,7 @@
         </is>
       </c>
       <c r="M105" t="inlineStr"/>
+      <c r="N105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7169,6 +7278,7 @@
       </c>
       <c r="L106" t="inlineStr"/>
       <c r="M106" t="inlineStr"/>
+      <c r="N106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -7220,6 +7330,7 @@
       </c>
       <c r="L107" t="inlineStr"/>
       <c r="M107" t="inlineStr"/>
+      <c r="N107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7271,6 +7382,7 @@
       </c>
       <c r="L108" t="inlineStr"/>
       <c r="M108" t="inlineStr"/>
+      <c r="N108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7322,6 +7434,7 @@
       </c>
       <c r="L109" t="inlineStr"/>
       <c r="M109" t="inlineStr"/>
+      <c r="N109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7373,6 +7486,7 @@
       </c>
       <c r="L110" t="inlineStr"/>
       <c r="M110" t="inlineStr"/>
+      <c r="N110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -7424,6 +7538,7 @@
       </c>
       <c r="L111" t="inlineStr"/>
       <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -7475,6 +7590,7 @@
       </c>
       <c r="L112" t="inlineStr"/>
       <c r="M112" t="inlineStr"/>
+      <c r="N112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -7526,6 +7642,7 @@
       </c>
       <c r="L113" t="inlineStr"/>
       <c r="M113" t="inlineStr"/>
+      <c r="N113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -7577,6 +7694,7 @@
       </c>
       <c r="L114" t="inlineStr"/>
       <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -7628,6 +7746,7 @@
       </c>
       <c r="L115" t="inlineStr"/>
       <c r="M115" t="inlineStr"/>
+      <c r="N115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -7679,6 +7798,7 @@
       </c>
       <c r="L116" t="inlineStr"/>
       <c r="M116" t="inlineStr"/>
+      <c r="N116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -7730,6 +7850,7 @@
       </c>
       <c r="L117" t="inlineStr"/>
       <c r="M117" t="inlineStr"/>
+      <c r="N117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -7781,6 +7902,7 @@
       </c>
       <c r="L118" t="inlineStr"/>
       <c r="M118" t="inlineStr"/>
+      <c r="N118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -7832,6 +7954,7 @@
       </c>
       <c r="L119" t="inlineStr"/>
       <c r="M119" t="inlineStr"/>
+      <c r="N119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7883,6 +8006,7 @@
       </c>
       <c r="L120" t="inlineStr"/>
       <c r="M120" t="inlineStr"/>
+      <c r="N120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7934,6 +8058,7 @@
       </c>
       <c r="L121" t="inlineStr"/>
       <c r="M121" t="inlineStr"/>
+      <c r="N121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7985,6 +8110,7 @@
       </c>
       <c r="L122" t="inlineStr"/>
       <c r="M122" t="inlineStr"/>
+      <c r="N122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8036,6 +8162,7 @@
       </c>
       <c r="L123" t="inlineStr"/>
       <c r="M123" t="inlineStr"/>
+      <c r="N123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8087,6 +8214,7 @@
       </c>
       <c r="L124" t="inlineStr"/>
       <c r="M124" t="inlineStr"/>
+      <c r="N124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -8138,6 +8266,7 @@
       </c>
       <c r="L125" t="inlineStr"/>
       <c r="M125" t="inlineStr"/>
+      <c r="N125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -8189,6 +8318,7 @@
       </c>
       <c r="L126" t="inlineStr"/>
       <c r="M126" t="inlineStr"/>
+      <c r="N126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -8240,6 +8370,7 @@
       </c>
       <c r="L127" t="inlineStr"/>
       <c r="M127" t="inlineStr"/>
+      <c r="N127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -8291,6 +8422,7 @@
       </c>
       <c r="L128" t="inlineStr"/>
       <c r="M128" t="inlineStr"/>
+      <c r="N128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -8342,6 +8474,7 @@
       </c>
       <c r="L129" t="inlineStr"/>
       <c r="M129" t="inlineStr"/>
+      <c r="N129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -8393,6 +8526,7 @@
       </c>
       <c r="L130" t="inlineStr"/>
       <c r="M130" t="inlineStr"/>
+      <c r="N130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -8444,6 +8578,7 @@
       </c>
       <c r="L131" t="inlineStr"/>
       <c r="M131" t="inlineStr"/>
+      <c r="N131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -8495,6 +8630,7 @@
       </c>
       <c r="L132" t="inlineStr"/>
       <c r="M132" t="inlineStr"/>
+      <c r="N132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -8546,6 +8682,7 @@
       </c>
       <c r="L133" t="inlineStr"/>
       <c r="M133" t="inlineStr"/>
+      <c r="N133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -8597,6 +8734,7 @@
       </c>
       <c r="L134" t="inlineStr"/>
       <c r="M134" t="inlineStr"/>
+      <c r="N134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -8648,6 +8786,7 @@
       </c>
       <c r="L135" t="inlineStr"/>
       <c r="M135" t="inlineStr"/>
+      <c r="N135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -8699,6 +8838,7 @@
       </c>
       <c r="L136" t="inlineStr"/>
       <c r="M136" t="inlineStr"/>
+      <c r="N136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -8750,6 +8890,7 @@
       </c>
       <c r="L137" t="inlineStr"/>
       <c r="M137" t="inlineStr"/>
+      <c r="N137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -8801,6 +8942,7 @@
       </c>
       <c r="L138" t="inlineStr"/>
       <c r="M138" t="inlineStr"/>
+      <c r="N138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -8856,6 +8998,7 @@
         </is>
       </c>
       <c r="M139" t="inlineStr"/>
+      <c r="N139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -8907,6 +9050,7 @@
       </c>
       <c r="L140" t="inlineStr"/>
       <c r="M140" t="inlineStr"/>
+      <c r="N140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -8958,6 +9102,7 @@
       </c>
       <c r="L141" t="inlineStr"/>
       <c r="M141" t="inlineStr"/>
+      <c r="N141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -9009,6 +9154,7 @@
       </c>
       <c r="L142" t="inlineStr"/>
       <c r="M142" t="inlineStr"/>
+      <c r="N142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -9060,6 +9206,7 @@
       </c>
       <c r="L143" t="inlineStr"/>
       <c r="M143" t="inlineStr"/>
+      <c r="N143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -9111,6 +9258,7 @@
       </c>
       <c r="L144" t="inlineStr"/>
       <c r="M144" t="inlineStr"/>
+      <c r="N144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -9162,6 +9310,7 @@
       </c>
       <c r="L145" t="inlineStr"/>
       <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -9213,6 +9362,7 @@
       </c>
       <c r="L146" t="inlineStr"/>
       <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -9264,6 +9414,7 @@
       </c>
       <c r="L147" t="inlineStr"/>
       <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -9315,6 +9466,7 @@
       </c>
       <c r="L148" t="inlineStr"/>
       <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -9366,6 +9518,7 @@
       </c>
       <c r="L149" t="inlineStr"/>
       <c r="M149" t="inlineStr"/>
+      <c r="N149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -9417,6 +9570,7 @@
       </c>
       <c r="L150" t="inlineStr"/>
       <c r="M150" t="inlineStr"/>
+      <c r="N150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -9468,6 +9622,7 @@
       </c>
       <c r="L151" t="inlineStr"/>
       <c r="M151" t="inlineStr"/>
+      <c r="N151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -9519,6 +9674,7 @@
       </c>
       <c r="L152" t="inlineStr"/>
       <c r="M152" t="inlineStr"/>
+      <c r="N152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -9570,6 +9726,7 @@
       </c>
       <c r="L153" t="inlineStr"/>
       <c r="M153" t="inlineStr"/>
+      <c r="N153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -9621,6 +9778,7 @@
       </c>
       <c r="L154" t="inlineStr"/>
       <c r="M154" t="inlineStr"/>
+      <c r="N154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -9672,6 +9830,7 @@
       </c>
       <c r="L155" t="inlineStr"/>
       <c r="M155" t="inlineStr"/>
+      <c r="N155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -9723,6 +9882,7 @@
       </c>
       <c r="L156" t="inlineStr"/>
       <c r="M156" t="inlineStr"/>
+      <c r="N156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -9774,6 +9934,7 @@
       </c>
       <c r="L157" t="inlineStr"/>
       <c r="M157" t="inlineStr"/>
+      <c r="N157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -9825,6 +9986,7 @@
       </c>
       <c r="L158" t="inlineStr"/>
       <c r="M158" t="inlineStr"/>
+      <c r="N158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -9876,6 +10038,7 @@
       </c>
       <c r="L159" t="inlineStr"/>
       <c r="M159" t="inlineStr"/>
+      <c r="N159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -9927,6 +10090,7 @@
       </c>
       <c r="L160" t="inlineStr"/>
       <c r="M160" t="inlineStr"/>
+      <c r="N160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -9978,6 +10142,7 @@
       </c>
       <c r="L161" t="inlineStr"/>
       <c r="M161" t="inlineStr"/>
+      <c r="N161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -10029,6 +10194,7 @@
       </c>
       <c r="L162" t="inlineStr"/>
       <c r="M162" t="inlineStr"/>
+      <c r="N162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -10080,6 +10246,7 @@
       </c>
       <c r="L163" t="inlineStr"/>
       <c r="M163" t="inlineStr"/>
+      <c r="N163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -10131,6 +10298,7 @@
       </c>
       <c r="L164" t="inlineStr"/>
       <c r="M164" t="inlineStr"/>
+      <c r="N164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -10182,6 +10350,7 @@
       </c>
       <c r="L165" t="inlineStr"/>
       <c r="M165" t="inlineStr"/>
+      <c r="N165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -10233,6 +10402,7 @@
       </c>
       <c r="L166" t="inlineStr"/>
       <c r="M166" t="inlineStr"/>
+      <c r="N166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -10284,6 +10454,7 @@
       </c>
       <c r="L167" t="inlineStr"/>
       <c r="M167" t="inlineStr"/>
+      <c r="N167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -10335,6 +10506,7 @@
       </c>
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="inlineStr"/>
+      <c r="N168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -10386,6 +10558,7 @@
       </c>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="inlineStr"/>
+      <c r="N169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -10437,6 +10610,7 @@
       </c>
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="inlineStr"/>
+      <c r="N170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -10488,6 +10662,7 @@
       </c>
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="inlineStr"/>
+      <c r="N171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -10539,6 +10714,7 @@
       </c>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="inlineStr"/>
+      <c r="N172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -10590,6 +10766,7 @@
       </c>
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -10645,6 +10822,7 @@
         </is>
       </c>
       <c r="M174" t="inlineStr"/>
+      <c r="N174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -10700,6 +10878,7 @@
         </is>
       </c>
       <c r="M175" t="inlineStr"/>
+      <c r="N175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -10751,6 +10930,7 @@
       </c>
       <c r="L176" t="inlineStr"/>
       <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -10802,6 +10982,7 @@
       </c>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -10853,6 +11034,7 @@
       </c>
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -10908,6 +11090,7 @@
         </is>
       </c>
       <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -10959,6 +11142,7 @@
       </c>
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -11014,6 +11198,7 @@
         </is>
       </c>
       <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -11065,6 +11250,7 @@
       </c>
       <c r="L182" t="inlineStr"/>
       <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -11116,6 +11302,7 @@
       </c>
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="inlineStr"/>
+      <c r="N183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -11167,6 +11354,7 @@
       </c>
       <c r="L184" t="inlineStr"/>
       <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -11218,6 +11406,7 @@
       </c>
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -11269,6 +11458,7 @@
       </c>
       <c r="L186" t="inlineStr"/>
       <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -11320,6 +11510,7 @@
       </c>
       <c r="L187" t="inlineStr"/>
       <c r="M187" t="inlineStr"/>
+      <c r="N187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -11371,6 +11562,7 @@
       </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="inlineStr"/>
+      <c r="N188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -11422,6 +11614,7 @@
       </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="inlineStr"/>
+      <c r="N189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -11473,6 +11666,7 @@
       </c>
       <c r="L190" t="inlineStr"/>
       <c r="M190" t="inlineStr"/>
+      <c r="N190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -11524,6 +11718,7 @@
       </c>
       <c r="L191" t="inlineStr"/>
       <c r="M191" t="inlineStr"/>
+      <c r="N191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -11575,6 +11770,7 @@
       </c>
       <c r="L192" t="inlineStr"/>
       <c r="M192" t="inlineStr"/>
+      <c r="N192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -11626,6 +11822,7 @@
       </c>
       <c r="L193" t="inlineStr"/>
       <c r="M193" t="inlineStr"/>
+      <c r="N193" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12251,7 +12448,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Food security: access and enabling factors</t>
+          <t>Food access and enabling factors</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">

</xml_diff>